<commit_message>
22 websites order form added
</commit_message>
<xml_diff>
--- a/data/currencyRates.xlsx
+++ b/data/currencyRates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CIT-23\Documents\CurrencyRateChecker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE497A4-A817-4074-933C-6318B7CA1CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3356495E-392F-4F5F-869D-9F1FD16D49E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F840A8F2-E93A-470D-A5EC-B9410A706CD1}"/>
   </bookViews>
@@ -452,7 +452,7 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>371.62</v>
+        <v>370.73</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -463,7 +463,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>319.8</v>
+        <v>318.02</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -474,7 +474,7 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>196.97</v>
+        <v>197.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>